<commit_message>
Dapine v3.0 - DuckDB disabled, Python engine faster (2.3s for 84 steps), all filters working
</commit_message>
<xml_diff>
--- a/ultimate_report.xlsx
+++ b/ultimate_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -434,7 +434,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,6 +472,56 @@
         <is>
           <t>avg_ppsf</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1350000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>450000</v>
+      </c>
+      <c r="E2" t="n">
+        <v>400000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>201.5151515151515</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1150000</v>
+      </c>
+      <c r="D3" t="n">
+        <v>575000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>550000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>600000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>198.2142857142857</v>
       </c>
     </row>
   </sheetData>

</xml_diff>